<commit_message>
Fixed some erros on the files
</commit_message>
<xml_diff>
--- a/akrami_Ex3A_tables.xlsx
+++ b/akrami_Ex3A_tables.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\sayaeedarashullahakr\Documents\DATA_Labs\W2_Workshop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AC699A50-A1E8-4264-A80E-97F69CE92929}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1ADDE020-A657-4075-A651-13D8B4A96634}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="3552" yWindow="3552" windowWidth="17280" windowHeight="9960" activeTab="3" xr2:uid="{1108299C-4170-418C-818F-0CB701B95CEF}"/>
   </bookViews>
@@ -16,7 +16,7 @@
     <sheet name="Client" sheetId="1" r:id="rId1"/>
     <sheet name="Dog" sheetId="2" r:id="rId2"/>
     <sheet name="Staff" sheetId="3" r:id="rId3"/>
-    <sheet name="Appointment" sheetId="4" r:id="rId4"/>
+    <sheet name="Appointments" sheetId="4" r:id="rId4"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>

</xml_diff>